<commit_message>
Add Sector Contribution Dofile
</commit_message>
<xml_diff>
--- a/data/raw/tfp.xlsx
+++ b/data/raw/tfp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desca\Documents\Island Economics\Consultancy\Belize-Labour-Assessment\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desca\Documents\Island Economics\Consultancy\Belize-Labour-Assessment\Data\Belize-Labour-Market-Analysis\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{726CB299-2765-4822-8BFE-FDC789311449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A04D055-80EE-4AA6-9114-3D56329EF994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C819B3D0-DFCD-4F57-932E-34D3CB349872}"/>
   </bookViews>
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -120,6 +120,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -572,6 +573,9 @@
       <c r="D12" s="4">
         <v>2.33295869827271</v>
       </c>
+      <c r="E12" s="6">
+        <v>123.06287902155425</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -586,6 +590,9 @@
       <c r="D13" s="3">
         <v>2.3458554744720499</v>
       </c>
+      <c r="E13" s="6">
+        <v>125.98241172715163</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -600,6 +607,9 @@
       <c r="D14" s="3">
         <v>2.3588235378265399</v>
       </c>
+      <c r="E14" s="6">
+        <v>101.93920121046736</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -614,6 +624,9 @@
       <c r="D15" s="3">
         <v>2.3718633651733398</v>
       </c>
+      <c r="E15" s="6">
+        <v>86.522965395337891</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -628,6 +641,9 @@
       <c r="D16" s="3">
         <v>2.3849751949310298</v>
       </c>
+      <c r="E16" s="6">
+        <v>102.81669064538283</v>
+      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
@@ -642,6 +658,9 @@
       <c r="D17" s="3">
         <v>2.3981595039367698</v>
       </c>
+      <c r="E17" s="6">
+        <v>87.822903315348412</v>
+      </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
@@ -656,6 +675,9 @@
       <c r="D18" s="3">
         <v>2.4407074451446502</v>
       </c>
+      <c r="E18" s="6">
+        <v>96.724406854398183</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
@@ -670,6 +692,9 @@
       <c r="D19" s="3">
         <v>2.4840099811553999</v>
       </c>
+      <c r="E19" s="6">
+        <v>141.8424064850812</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
@@ -684,6 +709,9 @@
       <c r="D20" s="3">
         <v>2.5280809402465798</v>
       </c>
+      <c r="E20" s="6">
+        <v>188.18262354296789</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
@@ -697,6 +725,9 @@
       </c>
       <c r="D21" s="3">
         <v>2.5686945915222199</v>
+      </c>
+      <c r="E21" s="6">
+        <v>220.72870668398321</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>